<commit_message>
tooltip mapping xlsx for atom and gas framework
</commit_message>
<xml_diff>
--- a/dataland-framework-toolbox/inputs/nuclear-and-gas/nuclear-and-gas.xlsx
+++ b/dataland-framework-toolbox/inputs/nuclear-and-gas/nuclear-and-gas.xlsx
@@ -5,15 +5,16 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\d93401\Projects\Dataland\dataland-framework-toolbox\inputs\nuclear-and-gas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\d92129\IdeaProjects\Dataland\dataland-framework-toolbox\inputs\nuclear-and-gas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:11_{B595F3C6-CB16-45A4-9A94-9BF24DD6B227}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2C263E5-B27E-4A4C-98AA-D1244248D238}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="33600" yWindow="2430" windowWidth="21600" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Framework Data Model" sheetId="1" r:id="rId1"/>
+    <sheet name="Tooltip Mapping" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="145621"/>
 </workbook>
@@ -624,18 +625,18 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:L173"/>
-  <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="7.453125" style="6" customWidth="1"/>
-    <col min="2" max="2" width="17.7265625" style="6" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" style="6" customWidth="1"/>
+    <col min="2" max="2" width="17.7109375" style="6" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" style="6" customWidth="1"/>
-    <col min="4" max="4" width="35.08984375" style="6" customWidth="1"/>
-    <col min="5" max="5" width="51.453125" style="6" customWidth="1"/>
+    <col min="4" max="4" width="35.140625" style="6" customWidth="1"/>
+    <col min="5" max="5" width="51.42578125" style="6" customWidth="1"/>
     <col min="6" max="12" width="15" style="6" customWidth="1"/>
-    <col min="13" max="16384" width="8.7265625" style="6"/>
+    <col min="13" max="16384" width="8.7109375" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="24" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="24" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -673,7 +674,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" s="7">
         <v>0</v>
       </c>
@@ -701,7 +702,7 @@
       <c r="K2" s="12"/>
       <c r="L2" s="12"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" s="7">
         <v>1</v>
       </c>
@@ -729,7 +730,7 @@
       <c r="K3" s="12"/>
       <c r="L3" s="12"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="7">
         <v>2</v>
       </c>
@@ -757,7 +758,7 @@
       <c r="K4" s="12"/>
       <c r="L4" s="12"/>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="7">
         <v>3</v>
       </c>
@@ -785,7 +786,7 @@
       <c r="K5" s="12"/>
       <c r="L5" s="12"/>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="7">
         <v>4</v>
       </c>
@@ -813,7 +814,7 @@
       <c r="K6" s="12"/>
       <c r="L6" s="12"/>
     </row>
-    <row r="7" spans="1:12" ht="13.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="13">
         <v>5</v>
       </c>
@@ -841,33 +842,42 @@
       <c r="K7" s="18"/>
       <c r="L7" s="18"/>
     </row>
-    <row r="145" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="145" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E145" s="8"/>
     </row>
-    <row r="146" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="146" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E146" s="8"/>
     </row>
-    <row r="147" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="147" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E147" s="8"/>
     </row>
-    <row r="148" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="148" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E148" s="8"/>
     </row>
-    <row r="170" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="170" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E170" s="8"/>
     </row>
-    <row r="171" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="171" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E171" s="8"/>
     </row>
-    <row r="172" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="172" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E172" s="8"/>
     </row>
-    <row r="173" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="173" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E173" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8998252D-8934-4923-BAE2-E6D038E56598}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -922,31 +932,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_dlc_DocId xmlns="fa7e5010-1311-4096-a344-326d1919664c">JFHTZT72FDVU-254938863-279</_dlc_DocId>
-    <_dlc_DocIdUrl xmlns="fa7e5010-1311-4096-a344-326d1919664c">
-      <Url>https://intranet.d-fine.de/intern/miscellaneous/TemplateFramework/_layouts/15/DocIdRedir.aspx?ID=JFHTZT72FDVU-254938863-279</Url>
-      <Description>JFHTZT72FDVU-254938863-279</Description>
-    </_dlc_DocIdUrl>
-    <_Version xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <Tools xmlns="255ceb00-0504-4451-971c-89cf8ee3ad27"/>
-    <Comments xmlns="255ceb00-0504-4451-971c-89cf8ee3ad27" xsi:nil="true"/>
-    <Document_x0020_Category xmlns="255ceb00-0504-4451-971c-89cf8ee3ad27"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100135AEE51B13C7A4784C7A6FB658DD0E0" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c2ccf66da846160ccad12796df698db1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="fa7e5010-1311-4096-a344-326d1919664c" xmlns:ns3="http://schemas.microsoft.com/sharepoint/v3/fields" xmlns:ns4="255ceb00-0504-4451-971c-89cf8ee3ad27" xmlns:ns5="953edb04-63dd-49ba-ad7b-e9d17e0e7f06" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="cd9e9067e801230649229059a2f6238c" ns2:_="" ns3:_="" ns4:_="" ns5:_="">
     <xsd:import namespace="fa7e5010-1311-4096-a344-326d1919664c"/>
@@ -1192,6 +1177,31 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_dlc_DocId xmlns="fa7e5010-1311-4096-a344-326d1919664c">JFHTZT72FDVU-254938863-279</_dlc_DocId>
+    <_dlc_DocIdUrl xmlns="fa7e5010-1311-4096-a344-326d1919664c">
+      <Url>https://intranet.d-fine.de/intern/miscellaneous/TemplateFramework/_layouts/15/DocIdRedir.aspx?ID=JFHTZT72FDVU-254938863-279</Url>
+      <Description>JFHTZT72FDVU-254938863-279</Description>
+    </_dlc_DocIdUrl>
+    <_Version xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <Tools xmlns="255ceb00-0504-4451-971c-89cf8ee3ad27"/>
+    <Comments xmlns="255ceb00-0504-4451-971c-89cf8ee3ad27" xsi:nil="true"/>
+    <Document_x0020_Category xmlns="255ceb00-0504-4451-971c-89cf8ee3ad27"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{27E0ED53-E837-41F7-A9C9-5E67E49390EA}">
   <ds:schemaRefs>
@@ -1201,9 +1211,22 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB0B7321-043A-43C5-BAA4-E29877D5579D}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FF6E80A2-72F6-4920-8A44-B99818E21D00}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="fa7e5010-1311-4096-a344-326d1919664c"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
+    <ds:schemaRef ds:uri="255ceb00-0504-4451-971c-89cf8ee3ad27"/>
+    <ds:schemaRef ds:uri="953edb04-63dd-49ba-ad7b-e9d17e0e7f06"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1228,22 +1251,9 @@
 </file>
 
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FF6E80A2-72F6-4920-8A44-B99818E21D00}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB0B7321-043A-43C5-BAA4-E29877D5579D}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="fa7e5010-1311-4096-a344-326d1919664c"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
-    <ds:schemaRef ds:uri="255ceb00-0504-4451-971c-89cf8ee3ad27"/>
-    <ds:schemaRef ds:uri="953edb04-63dd-49ba-ad7b-e9d17e0e7f06"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
first version of framework in framework custom component
</commit_message>
<xml_diff>
--- a/dataland-framework-toolbox/inputs/nuclear-and-gas/nuclear-and-gas.xlsx
+++ b/dataland-framework-toolbox/inputs/nuclear-and-gas/nuclear-and-gas.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\d93401\Documents\Dataland\Taxonomy and Frameworks\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\d93447\Documents\Dataland\dataland-framework-toolbox\inputs\nuclear-and-gas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90549E64-1797-4597-9727-16D08DABC138}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B687165E-F597-4C45-8B03-3F52709B52F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="1725" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1193" yWindow="442" windowWidth="26242" windowHeight="14761" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Framework Data Model" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="238">
   <si>
     <t>Field Identifier</t>
   </si>
@@ -86,9 +86,6 @@
     <t>The undertaking carries out, funds, or has exposures to construction, refurbishment and operation of heat generation facilities that produce heat/cool using fossil gaseous fuels.</t>
   </si>
   <si>
-    <t>CustomComponent</t>
-  </si>
-  <si>
     <t>Template</t>
   </si>
   <si>
@@ -726,6 +723,18 @@
   </si>
   <si>
     <t>Proportion of Taxonomy-non-eligible Economic Activity referred to in Sections 4.26 to 4.31 of Annexes I and II to Delegated Regulation 2021/2139 in the numerator of the applicable KPI - Revenue-based</t>
+  </si>
+  <si>
+    <t>CustomComponent Aligned (Denominator)</t>
+  </si>
+  <si>
+    <t>CustomComponent Aligned (Numerator)</t>
+  </si>
+  <si>
+    <t>CustomComponent Eligible but not aligned</t>
+  </si>
+  <si>
+    <t>CustomComponent Non-Eligible</t>
   </si>
 </sst>
 </file>
@@ -1466,19 +1475,19 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:L173"/>
-  <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="13.15" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="7.453125" style="4" customWidth="1"/>
-    <col min="2" max="2" width="17.7265625" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15" style="4" customWidth="1"/>
-    <col min="4" max="4" width="41.453125" style="4" customWidth="1"/>
-    <col min="5" max="5" width="143.90625" style="4" customWidth="1"/>
-    <col min="6" max="6" width="15.7265625" style="4" customWidth="1"/>
+    <col min="1" max="1" width="7.46484375" style="4" customWidth="1"/>
+    <col min="2" max="2" width="17.73046875" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.86328125" style="4" customWidth="1"/>
+    <col min="4" max="4" width="41.46484375" style="4" customWidth="1"/>
+    <col min="5" max="5" width="45.73046875" style="4" customWidth="1"/>
+    <col min="6" max="6" width="32.6640625" style="4" customWidth="1"/>
     <col min="7" max="12" width="15" style="4" customWidth="1"/>
-    <col min="13" max="16384" width="8.7265625" style="4"/>
+    <col min="13" max="16384" width="8.73046875" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="24" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="23.25" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1516,7 +1525,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A2" s="44">
         <v>1</v>
       </c>
@@ -1524,10 +1533,10 @@
         <v>14</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D2" s="22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E2" s="22" t="s">
         <v>15</v>
@@ -1544,7 +1553,7 @@
       <c r="K2" s="24"/>
       <c r="L2" s="24"/>
     </row>
-    <row r="3" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A3" s="44">
         <v>2</v>
       </c>
@@ -1552,10 +1561,10 @@
         <v>14</v>
       </c>
       <c r="C3" s="21" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D3" s="22" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E3" s="22" t="s">
         <v>16</v>
@@ -1572,7 +1581,7 @@
       <c r="K3" s="24"/>
       <c r="L3" s="24"/>
     </row>
-    <row r="4" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A4" s="44">
         <v>3</v>
       </c>
@@ -1580,10 +1589,10 @@
         <v>14</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D4" s="22" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E4" s="22" t="s">
         <v>17</v>
@@ -1600,7 +1609,7 @@
       <c r="K4" s="24"/>
       <c r="L4" s="24"/>
     </row>
-    <row r="5" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A5" s="44">
         <v>4</v>
       </c>
@@ -1608,10 +1617,10 @@
         <v>14</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D5" s="22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E5" s="22" t="s">
         <v>18</v>
@@ -1628,7 +1637,7 @@
       <c r="K5" s="24"/>
       <c r="L5" s="24"/>
     </row>
-    <row r="6" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A6" s="44">
         <v>5</v>
       </c>
@@ -1636,10 +1645,10 @@
         <v>14</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D6" s="22" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E6" s="22" t="s">
         <v>19</v>
@@ -1656,7 +1665,7 @@
       <c r="K6" s="24"/>
       <c r="L6" s="24"/>
     </row>
-    <row r="7" spans="1:12" s="32" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" s="32" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A7" s="45">
         <v>6</v>
       </c>
@@ -1664,10 +1673,10 @@
         <v>14</v>
       </c>
       <c r="C7" s="28" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D7" s="29" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E7" s="29" t="s">
         <v>20</v>
@@ -1684,7 +1693,7 @@
       <c r="K7" s="31"/>
       <c r="L7" s="31"/>
     </row>
-    <row r="8" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A8" s="44">
         <v>7</v>
       </c>
@@ -1692,16 +1701,16 @@
         <v>14</v>
       </c>
       <c r="C8" s="21" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D8" s="33" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="E8" s="34" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F8" s="35" t="s">
-        <v>21</v>
+        <v>234</v>
       </c>
       <c r="G8" s="35"/>
       <c r="H8" s="36"/>
@@ -1712,7 +1721,7 @@
       <c r="K8" s="36"/>
       <c r="L8" s="36"/>
     </row>
-    <row r="9" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A9" s="44">
         <v>8</v>
       </c>
@@ -1720,16 +1729,16 @@
         <v>14</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D9" s="33" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E9" s="34" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F9" s="23" t="s">
-        <v>21</v>
+        <v>234</v>
       </c>
       <c r="G9" s="23"/>
       <c r="H9" s="24"/>
@@ -1740,7 +1749,7 @@
       <c r="K9" s="24"/>
       <c r="L9" s="24"/>
     </row>
-    <row r="10" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A10" s="44">
         <v>9</v>
       </c>
@@ -1748,16 +1757,16 @@
         <v>14</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D10" s="33" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E10" s="34" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="F10" s="23" t="s">
-        <v>21</v>
+        <v>235</v>
       </c>
       <c r="G10" s="23"/>
       <c r="H10" s="24"/>
@@ -1768,7 +1777,7 @@
       <c r="K10" s="24"/>
       <c r="L10" s="24"/>
     </row>
-    <row r="11" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A11" s="44">
         <v>10</v>
       </c>
@@ -1776,16 +1785,16 @@
         <v>14</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D11" s="33" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E11" s="34" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="F11" s="23" t="s">
-        <v>21</v>
+        <v>235</v>
       </c>
       <c r="G11" s="26"/>
       <c r="H11" s="24"/>
@@ -1796,7 +1805,7 @@
       <c r="K11" s="24"/>
       <c r="L11" s="24"/>
     </row>
-    <row r="12" spans="1:12" s="25" customFormat="1" ht="23" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" s="25" customFormat="1" ht="23.25" x14ac:dyDescent="0.4">
       <c r="A12" s="44">
         <v>11</v>
       </c>
@@ -1804,16 +1813,16 @@
         <v>14</v>
       </c>
       <c r="C12" s="21" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D12" s="33" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E12" s="38" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F12" s="39" t="s">
-        <v>21</v>
+        <v>236</v>
       </c>
       <c r="G12" s="39"/>
       <c r="H12" s="40"/>
@@ -1824,7 +1833,7 @@
       <c r="K12" s="40"/>
       <c r="L12" s="40"/>
     </row>
-    <row r="13" spans="1:12" s="25" customFormat="1" ht="23" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" s="25" customFormat="1" ht="23.25" x14ac:dyDescent="0.4">
       <c r="A13" s="44">
         <v>12</v>
       </c>
@@ -1832,16 +1841,16 @@
         <v>14</v>
       </c>
       <c r="C13" s="21" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D13" s="33" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E13" s="38" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F13" s="23" t="s">
-        <v>21</v>
+        <v>236</v>
       </c>
       <c r="G13" s="23"/>
       <c r="H13" s="24"/>
@@ -1852,7 +1861,7 @@
       <c r="K13" s="24"/>
       <c r="L13" s="24"/>
     </row>
-    <row r="14" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A14" s="44">
         <v>13</v>
       </c>
@@ -1860,16 +1869,16 @@
         <v>14</v>
       </c>
       <c r="C14" s="21" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D14" s="33" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E14" s="34" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F14" s="23" t="s">
-        <v>21</v>
+        <v>237</v>
       </c>
       <c r="G14" s="23"/>
       <c r="H14" s="24"/>
@@ -1880,7 +1889,7 @@
       <c r="K14" s="24"/>
       <c r="L14" s="24"/>
     </row>
-    <row r="15" spans="1:12" s="32" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" s="32" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A15" s="45">
         <v>14</v>
       </c>
@@ -1888,16 +1897,16 @@
         <v>14</v>
       </c>
       <c r="C15" s="42" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D15" s="43" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E15" s="34" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F15" s="30" t="s">
-        <v>21</v>
+        <v>237</v>
       </c>
       <c r="G15" s="30"/>
       <c r="H15" s="31"/>
@@ -1908,7 +1917,7 @@
       <c r="K15" s="31"/>
       <c r="L15" s="31"/>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A16"/>
       <c r="B16"/>
       <c r="C16"/>
@@ -1922,7 +1931,7 @@
       <c r="K16"/>
       <c r="L16"/>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A17"/>
       <c r="B17"/>
       <c r="C17"/>
@@ -1936,7 +1945,7 @@
       <c r="K17"/>
       <c r="L17"/>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A18"/>
       <c r="B18"/>
       <c r="C18"/>
@@ -1950,7 +1959,7 @@
       <c r="K18"/>
       <c r="L18"/>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A19"/>
       <c r="B19"/>
       <c r="C19"/>
@@ -1964,7 +1973,7 @@
       <c r="K19"/>
       <c r="L19"/>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A20"/>
       <c r="B20"/>
       <c r="C20"/>
@@ -1978,7 +1987,7 @@
       <c r="K20"/>
       <c r="L20"/>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A21"/>
       <c r="B21"/>
       <c r="C21"/>
@@ -1992,28 +2001,28 @@
       <c r="K21"/>
       <c r="L21"/>
     </row>
-    <row r="145" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="145" spans="5:5" x14ac:dyDescent="0.4">
       <c r="E145" s="5"/>
     </row>
-    <row r="146" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="146" spans="5:5" x14ac:dyDescent="0.4">
       <c r="E146" s="5"/>
     </row>
-    <row r="147" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="147" spans="5:5" x14ac:dyDescent="0.4">
       <c r="E147" s="5"/>
     </row>
-    <row r="148" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="148" spans="5:5" x14ac:dyDescent="0.4">
       <c r="E148" s="5"/>
     </row>
-    <row r="170" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="170" spans="5:5" x14ac:dyDescent="0.4">
       <c r="E170" s="5"/>
     </row>
-    <row r="171" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="171" spans="5:5" x14ac:dyDescent="0.4">
       <c r="E171" s="5"/>
     </row>
-    <row r="172" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="172" spans="5:5" x14ac:dyDescent="0.4">
       <c r="E172" s="5"/>
     </row>
-    <row r="173" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="173" spans="5:5" x14ac:dyDescent="0.4">
       <c r="E173" s="5"/>
     </row>
   </sheetData>
@@ -2025,22 +2034,22 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C899FC4-CD15-4806-A04E-7A6BABA59C0A}">
   <dimension ref="A1:K173"/>
-  <sheetFormatPr defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="14.55" customHeight="1" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="7.08984375" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.08984375" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="99.90625" style="4" customWidth="1"/>
-    <col min="4" max="4" width="119.36328125" style="4" customWidth="1"/>
+    <col min="1" max="1" width="7.06640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.06640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="99.9296875" style="4" customWidth="1"/>
+    <col min="4" max="4" width="119.33203125" style="4" customWidth="1"/>
     <col min="5" max="11" width="15" style="4" customWidth="1"/>
-    <col min="12" max="16384" width="8.7265625" style="4"/>
+    <col min="12" max="16384" width="8.73046875" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>3</v>
@@ -2070,21 +2079,21 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="9">
         <v>1</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C2" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F2" s="3"/>
       <c r="G2" s="6"/>
@@ -2093,21 +2102,21 @@
       <c r="J2" s="6"/>
       <c r="K2" s="6"/>
     </row>
-    <row r="3" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" s="9">
         <v>2</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F3" s="3"/>
       <c r="G3" s="6"/>
@@ -2116,21 +2125,21 @@
       <c r="J3" s="6"/>
       <c r="K3" s="6"/>
     </row>
-    <row r="4" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="9">
         <v>3</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F4" s="3"/>
       <c r="G4" s="6"/>
@@ -2139,21 +2148,21 @@
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
     </row>
-    <row r="5" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="9">
         <v>4</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="6"/>
@@ -2162,21 +2171,21 @@
       <c r="J5" s="6"/>
       <c r="K5" s="6"/>
     </row>
-    <row r="6" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="9">
         <v>5</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F6" s="3"/>
       <c r="G6" s="6"/>
@@ -2185,21 +2194,21 @@
       <c r="J6" s="6"/>
       <c r="K6" s="6"/>
     </row>
-    <row r="7" spans="1:11" s="11" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" s="11" customFormat="1" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="9">
         <v>6</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F7" s="3"/>
       <c r="G7" s="6"/>
@@ -2208,21 +2217,21 @@
       <c r="J7" s="6"/>
       <c r="K7" s="6"/>
     </row>
-    <row r="8" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A8" s="9">
         <v>7</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F8" s="3"/>
       <c r="G8" s="6"/>
@@ -2231,21 +2240,21 @@
       <c r="J8" s="6"/>
       <c r="K8" s="6"/>
     </row>
-    <row r="9" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="9">
         <v>8</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F9" s="3"/>
       <c r="G9" s="6"/>
@@ -2254,21 +2263,21 @@
       <c r="J9" s="6"/>
       <c r="K9" s="6"/>
     </row>
-    <row r="10" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A10" s="9">
         <v>9</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F10" s="3"/>
       <c r="G10" s="6"/>
@@ -2277,21 +2286,21 @@
       <c r="J10" s="6"/>
       <c r="K10" s="6"/>
     </row>
-    <row r="11" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A11" s="9">
         <v>10</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F11" s="3"/>
       <c r="G11" s="6"/>
@@ -2300,21 +2309,21 @@
       <c r="J11" s="6"/>
       <c r="K11" s="6"/>
     </row>
-    <row r="12" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A12" s="9">
         <v>11</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F12" s="3"/>
       <c r="G12" s="6"/>
@@ -2323,21 +2332,21 @@
       <c r="J12" s="6"/>
       <c r="K12" s="6"/>
     </row>
-    <row r="13" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A13" s="9">
         <v>12</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D13" s="17" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F13" s="3"/>
       <c r="G13" s="6"/>
@@ -2346,21 +2355,21 @@
       <c r="J13" s="6"/>
       <c r="K13" s="6"/>
     </row>
-    <row r="14" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A14" s="9">
         <v>13</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F14" s="3"/>
       <c r="G14" s="6"/>
@@ -2369,21 +2378,21 @@
       <c r="J14" s="6"/>
       <c r="K14" s="6"/>
     </row>
-    <row r="15" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A15" s="9">
         <v>14</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D15" s="17" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F15" s="3"/>
       <c r="G15" s="6"/>
@@ -2392,21 +2401,21 @@
       <c r="J15" s="6"/>
       <c r="K15" s="6"/>
     </row>
-    <row r="16" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A16" s="9">
         <v>15</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C16" s="16" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D16" s="17" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F16" s="3"/>
       <c r="G16" s="6"/>
@@ -2415,21 +2424,21 @@
       <c r="J16" s="6"/>
       <c r="K16" s="6"/>
     </row>
-    <row r="17" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A17" s="9">
         <v>16</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D17" s="17" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F17" s="3"/>
       <c r="G17" s="6"/>
@@ -2438,21 +2447,21 @@
       <c r="J17" s="6"/>
       <c r="K17" s="6"/>
     </row>
-    <row r="18" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A18" s="9">
         <v>17</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D18" s="17" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F18" s="3"/>
       <c r="G18" s="6"/>
@@ -2461,21 +2470,21 @@
       <c r="J18" s="6"/>
       <c r="K18" s="6"/>
     </row>
-    <row r="19" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A19" s="9">
         <v>18</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C19" s="16" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D19" s="17" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F19" s="3"/>
       <c r="G19" s="6"/>
@@ -2484,21 +2493,21 @@
       <c r="J19" s="6"/>
       <c r="K19" s="6"/>
     </row>
-    <row r="20" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A20" s="9">
         <v>19</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C20" s="16" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D20" s="17" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F20" s="3"/>
       <c r="G20" s="6"/>
@@ -2507,21 +2516,21 @@
       <c r="J20" s="6"/>
       <c r="K20" s="6"/>
     </row>
-    <row r="21" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A21" s="9">
         <v>20</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D21" s="17" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F21" s="3"/>
       <c r="G21" s="6"/>
@@ -2530,21 +2539,21 @@
       <c r="J21" s="6"/>
       <c r="K21" s="6"/>
     </row>
-    <row r="22" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A22" s="9">
         <v>21</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C22" s="16" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D22" s="17" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F22" s="3"/>
       <c r="G22" s="6"/>
@@ -2553,21 +2562,21 @@
       <c r="J22" s="6"/>
       <c r="K22" s="6"/>
     </row>
-    <row r="23" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A23" s="9">
         <v>22</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D23" s="16" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F23" s="3"/>
       <c r="G23" s="6"/>
@@ -2576,21 +2585,21 @@
       <c r="J23" s="6"/>
       <c r="K23" s="6"/>
     </row>
-    <row r="24" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A24" s="9">
         <v>23</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C24" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="D24" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="D24" s="16" t="s">
-        <v>41</v>
-      </c>
       <c r="E24" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F24" s="3"/>
       <c r="G24" s="6"/>
@@ -2599,21 +2608,21 @@
       <c r="J24" s="6"/>
       <c r="K24" s="6"/>
     </row>
-    <row r="25" spans="1:11" s="10" customFormat="1" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" s="10" customFormat="1" ht="14.55" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A25" s="14">
         <v>24</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C25" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="D25" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="D25" s="19" t="s">
-        <v>50</v>
-      </c>
       <c r="E25" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F25" s="7"/>
       <c r="G25" s="8"/>
@@ -2622,21 +2631,21 @@
       <c r="J25" s="8"/>
       <c r="K25" s="8"/>
     </row>
-    <row r="26" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A26" s="9">
         <v>25</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C26" s="16" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D26" s="17" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F26" s="3"/>
       <c r="G26" s="6"/>
@@ -2645,21 +2654,21 @@
       <c r="J26" s="6"/>
       <c r="K26" s="6"/>
     </row>
-    <row r="27" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A27" s="9">
         <v>26</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C27" s="16" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D27" s="17" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F27" s="3"/>
       <c r="G27" s="6"/>
@@ -2668,21 +2677,21 @@
       <c r="J27" s="6"/>
       <c r="K27" s="6"/>
     </row>
-    <row r="28" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A28" s="9">
         <v>27</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C28" s="16" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D28" s="17" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F28" s="3"/>
       <c r="G28" s="6"/>
@@ -2691,21 +2700,21 @@
       <c r="J28" s="6"/>
       <c r="K28" s="6"/>
     </row>
-    <row r="29" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A29" s="9">
         <v>28</v>
       </c>
       <c r="B29" s="13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C29" s="16" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D29" s="17" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F29" s="2"/>
       <c r="G29" s="6"/>
@@ -2714,21 +2723,21 @@
       <c r="J29" s="6"/>
       <c r="K29" s="6"/>
     </row>
-    <row r="30" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A30" s="9">
         <v>29</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C30" s="16" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D30" s="17" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F30" s="3"/>
       <c r="G30" s="6"/>
@@ -2737,21 +2746,21 @@
       <c r="J30" s="6"/>
       <c r="K30" s="6"/>
     </row>
-    <row r="31" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A31" s="9">
         <v>30</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C31" s="16" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D31" s="17" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F31" s="3"/>
       <c r="G31" s="6"/>
@@ -2760,21 +2769,21 @@
       <c r="J31" s="6"/>
       <c r="K31" s="6"/>
     </row>
-    <row r="32" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A32" s="9">
         <v>31</v>
       </c>
       <c r="B32" s="13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C32" s="16" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D32" s="17" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F32" s="3"/>
       <c r="G32" s="6"/>
@@ -2783,21 +2792,21 @@
       <c r="J32" s="6"/>
       <c r="K32" s="6"/>
     </row>
-    <row r="33" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A33" s="9">
         <v>32</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C33" s="16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D33" s="17" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F33" s="3"/>
       <c r="G33" s="6"/>
@@ -2806,21 +2815,21 @@
       <c r="J33" s="6"/>
       <c r="K33" s="6"/>
     </row>
-    <row r="34" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A34" s="9">
         <v>33</v>
       </c>
       <c r="B34" s="13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D34" s="17" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F34" s="3"/>
       <c r="G34" s="6"/>
@@ -2829,21 +2838,21 @@
       <c r="J34" s="6"/>
       <c r="K34" s="6"/>
     </row>
-    <row r="35" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A35" s="9">
         <v>34</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C35" s="16" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D35" s="17" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F35" s="3"/>
       <c r="G35" s="6"/>
@@ -2852,21 +2861,21 @@
       <c r="J35" s="6"/>
       <c r="K35" s="6"/>
     </row>
-    <row r="36" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A36" s="9">
         <v>35</v>
       </c>
       <c r="B36" s="13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C36" s="16" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D36" s="17" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F36" s="3"/>
       <c r="G36" s="6"/>
@@ -2875,21 +2884,21 @@
       <c r="J36" s="6"/>
       <c r="K36" s="6"/>
     </row>
-    <row r="37" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A37" s="9">
         <v>36</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C37" s="16" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D37" s="17" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F37" s="3"/>
       <c r="G37" s="6"/>
@@ -2898,21 +2907,21 @@
       <c r="J37" s="6"/>
       <c r="K37" s="6"/>
     </row>
-    <row r="38" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A38" s="9">
         <v>37</v>
       </c>
       <c r="B38" s="13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C38" s="16" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D38" s="17" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F38" s="3"/>
       <c r="G38" s="6"/>
@@ -2921,21 +2930,21 @@
       <c r="J38" s="6"/>
       <c r="K38" s="6"/>
     </row>
-    <row r="39" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A39" s="9">
         <v>38</v>
       </c>
       <c r="B39" s="13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C39" s="16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D39" s="17" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F39" s="3"/>
       <c r="G39" s="6"/>
@@ -2944,21 +2953,21 @@
       <c r="J39" s="6"/>
       <c r="K39" s="6"/>
     </row>
-    <row r="40" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A40" s="9">
         <v>39</v>
       </c>
       <c r="B40" s="13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C40" s="16" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D40" s="17" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F40" s="3"/>
       <c r="G40" s="6"/>
@@ -2967,21 +2976,21 @@
       <c r="J40" s="6"/>
       <c r="K40" s="6"/>
     </row>
-    <row r="41" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A41" s="9">
         <v>40</v>
       </c>
       <c r="B41" s="13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C41" s="16" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D41" s="17" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F41" s="3"/>
       <c r="G41" s="6"/>
@@ -2990,21 +2999,21 @@
       <c r="J41" s="6"/>
       <c r="K41" s="6"/>
     </row>
-    <row r="42" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A42" s="9">
         <v>41</v>
       </c>
       <c r="B42" s="13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C42" s="16" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D42" s="17" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F42" s="3"/>
       <c r="G42" s="6"/>
@@ -3013,21 +3022,21 @@
       <c r="J42" s="6"/>
       <c r="K42" s="6"/>
     </row>
-    <row r="43" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A43" s="9">
         <v>42</v>
       </c>
       <c r="B43" s="13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C43" s="16" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D43" s="17" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F43" s="3"/>
       <c r="G43" s="6"/>
@@ -3036,21 +3045,21 @@
       <c r="J43" s="6"/>
       <c r="K43" s="6"/>
     </row>
-    <row r="44" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A44" s="9">
         <v>43</v>
       </c>
       <c r="B44" s="13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D44" s="17" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F44" s="3"/>
       <c r="G44" s="6"/>
@@ -3059,21 +3068,21 @@
       <c r="J44" s="6"/>
       <c r="K44" s="6"/>
     </row>
-    <row r="45" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A45" s="9">
         <v>44</v>
       </c>
       <c r="B45" s="13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C45" s="16" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D45" s="17" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F45" s="3"/>
       <c r="G45" s="6"/>
@@ -3082,21 +3091,21 @@
       <c r="J45" s="6"/>
       <c r="K45" s="6"/>
     </row>
-    <row r="46" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A46" s="9">
         <v>45</v>
       </c>
       <c r="B46" s="13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C46" s="16" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D46" s="17" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F46" s="3"/>
       <c r="G46" s="6"/>
@@ -3105,21 +3114,21 @@
       <c r="J46" s="6"/>
       <c r="K46" s="6"/>
     </row>
-    <row r="47" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A47" s="9">
         <v>46</v>
       </c>
       <c r="B47" s="13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C47" s="16" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D47" s="16" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F47" s="3"/>
       <c r="G47" s="6"/>
@@ -3128,21 +3137,21 @@
       <c r="J47" s="6"/>
       <c r="K47" s="6"/>
     </row>
-    <row r="48" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A48" s="9">
         <v>47</v>
       </c>
       <c r="B48" s="13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C48" s="16" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D48" s="16" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F48" s="3"/>
       <c r="G48" s="6"/>
@@ -3151,21 +3160,21 @@
       <c r="J48" s="6"/>
       <c r="K48" s="6"/>
     </row>
-    <row r="49" spans="1:11" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:11" ht="14.55" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A49" s="14">
         <v>48</v>
       </c>
       <c r="B49" s="15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C49" s="18" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D49" s="19" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E49" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F49" s="7"/>
       <c r="G49" s="8"/>
@@ -3174,21 +3183,21 @@
       <c r="J49" s="8"/>
       <c r="K49" s="8"/>
     </row>
-    <row r="50" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A50" s="9">
         <v>49</v>
       </c>
       <c r="B50" s="12" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C50" s="16" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D50" s="17" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F50" s="3"/>
       <c r="G50" s="6"/>
@@ -3197,21 +3206,21 @@
       <c r="J50" s="6"/>
       <c r="K50" s="6"/>
     </row>
-    <row r="51" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A51" s="9">
         <v>50</v>
       </c>
       <c r="B51" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C51" s="16" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D51" s="17" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F51" s="3"/>
       <c r="G51" s="6"/>
@@ -3220,21 +3229,21 @@
       <c r="J51" s="6"/>
       <c r="K51" s="6"/>
     </row>
-    <row r="52" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A52" s="9">
         <v>51</v>
       </c>
       <c r="B52" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C52" s="16" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D52" s="17" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F52" s="3"/>
       <c r="G52" s="6"/>
@@ -3243,21 +3252,21 @@
       <c r="J52" s="6"/>
       <c r="K52" s="6"/>
     </row>
-    <row r="53" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A53" s="9">
         <v>52</v>
       </c>
       <c r="B53" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C53" s="16" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D53" s="17" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F53" s="2"/>
       <c r="G53" s="6"/>
@@ -3266,21 +3275,21 @@
       <c r="J53" s="6"/>
       <c r="K53" s="6"/>
     </row>
-    <row r="54" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A54" s="9">
         <v>53</v>
       </c>
       <c r="B54" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C54" s="16" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D54" s="17" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F54" s="3"/>
       <c r="G54" s="6"/>
@@ -3289,21 +3298,21 @@
       <c r="J54" s="6"/>
       <c r="K54" s="6"/>
     </row>
-    <row r="55" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A55" s="9">
         <v>54</v>
       </c>
       <c r="B55" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C55" s="16" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D55" s="17" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F55" s="3"/>
       <c r="G55" s="6"/>
@@ -3312,21 +3321,21 @@
       <c r="J55" s="6"/>
       <c r="K55" s="6"/>
     </row>
-    <row r="56" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A56" s="9">
         <v>55</v>
       </c>
       <c r="B56" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C56" s="16" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D56" s="17" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F56" s="3"/>
       <c r="G56" s="6"/>
@@ -3335,21 +3344,21 @@
       <c r="J56" s="6"/>
       <c r="K56" s="6"/>
     </row>
-    <row r="57" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A57" s="9">
         <v>56</v>
       </c>
       <c r="B57" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C57" s="16" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D57" s="17" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F57" s="3"/>
       <c r="G57" s="6"/>
@@ -3358,21 +3367,21 @@
       <c r="J57" s="6"/>
       <c r="K57" s="6"/>
     </row>
-    <row r="58" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A58" s="9">
         <v>57</v>
       </c>
       <c r="B58" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C58" s="16" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D58" s="17" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F58" s="3"/>
       <c r="G58" s="6"/>
@@ -3381,21 +3390,21 @@
       <c r="J58" s="6"/>
       <c r="K58" s="6"/>
     </row>
-    <row r="59" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A59" s="9">
         <v>58</v>
       </c>
       <c r="B59" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C59" s="16" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D59" s="17" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F59" s="3"/>
       <c r="G59" s="6"/>
@@ -3404,21 +3413,21 @@
       <c r="J59" s="6"/>
       <c r="K59" s="6"/>
     </row>
-    <row r="60" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A60" s="9">
         <v>59</v>
       </c>
       <c r="B60" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C60" s="16" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D60" s="17" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F60" s="3"/>
       <c r="G60" s="6"/>
@@ -3427,21 +3436,21 @@
       <c r="J60" s="6"/>
       <c r="K60" s="6"/>
     </row>
-    <row r="61" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A61" s="9">
         <v>60</v>
       </c>
       <c r="B61" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C61" s="16" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D61" s="17" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F61" s="3"/>
       <c r="G61" s="6"/>
@@ -3450,21 +3459,21 @@
       <c r="J61" s="6"/>
       <c r="K61" s="6"/>
     </row>
-    <row r="62" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A62" s="9">
         <v>61</v>
       </c>
       <c r="B62" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C62" s="16" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D62" s="17" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E62" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F62" s="3"/>
       <c r="G62" s="6"/>
@@ -3473,21 +3482,21 @@
       <c r="J62" s="6"/>
       <c r="K62" s="6"/>
     </row>
-    <row r="63" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A63" s="9">
         <v>62</v>
       </c>
       <c r="B63" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C63" s="16" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D63" s="17" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F63" s="3"/>
       <c r="G63" s="6"/>
@@ -3496,21 +3505,21 @@
       <c r="J63" s="6"/>
       <c r="K63" s="6"/>
     </row>
-    <row r="64" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A64" s="9">
         <v>63</v>
       </c>
       <c r="B64" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C64" s="16" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D64" s="17" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F64" s="3"/>
       <c r="G64" s="6"/>
@@ -3519,21 +3528,21 @@
       <c r="J64" s="6"/>
       <c r="K64" s="6"/>
     </row>
-    <row r="65" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A65" s="9">
         <v>64</v>
       </c>
       <c r="B65" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C65" s="16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D65" s="17" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E65" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F65" s="3"/>
       <c r="G65" s="6"/>
@@ -3542,21 +3551,21 @@
       <c r="J65" s="6"/>
       <c r="K65" s="6"/>
     </row>
-    <row r="66" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A66" s="9">
         <v>65</v>
       </c>
       <c r="B66" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C66" s="16" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D66" s="17" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="E66" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F66" s="3"/>
       <c r="G66" s="6"/>
@@ -3565,21 +3574,21 @@
       <c r="J66" s="6"/>
       <c r="K66" s="6"/>
     </row>
-    <row r="67" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A67" s="9">
         <v>66</v>
       </c>
       <c r="B67" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C67" s="16" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D67" s="17" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E67" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F67" s="3"/>
       <c r="G67" s="6"/>
@@ -3588,21 +3597,21 @@
       <c r="J67" s="6"/>
       <c r="K67" s="6"/>
     </row>
-    <row r="68" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A68" s="9">
         <v>67</v>
       </c>
       <c r="B68" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C68" s="16" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D68" s="17" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E68" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F68" s="3"/>
       <c r="G68" s="6"/>
@@ -3611,21 +3620,21 @@
       <c r="J68" s="6"/>
       <c r="K68" s="6"/>
     </row>
-    <row r="69" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A69" s="9">
         <v>68</v>
       </c>
       <c r="B69" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C69" s="16" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D69" s="17" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E69" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F69" s="3"/>
       <c r="G69" s="6"/>
@@ -3634,21 +3643,21 @@
       <c r="J69" s="6"/>
       <c r="K69" s="6"/>
     </row>
-    <row r="70" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A70" s="9">
         <v>69</v>
       </c>
       <c r="B70" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C70" s="16" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D70" s="17" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E70" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F70" s="3"/>
       <c r="G70" s="6"/>
@@ -3657,21 +3666,21 @@
       <c r="J70" s="6"/>
       <c r="K70" s="6"/>
     </row>
-    <row r="71" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A71" s="9">
         <v>70</v>
       </c>
       <c r="B71" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C71" s="16" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D71" s="16" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E71" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F71" s="3"/>
       <c r="G71" s="6"/>
@@ -3680,21 +3689,21 @@
       <c r="J71" s="6"/>
       <c r="K71" s="6"/>
     </row>
-    <row r="72" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A72" s="9">
         <v>71</v>
       </c>
       <c r="B72" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C72" s="16" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D72" s="16" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="E72" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F72" s="3"/>
       <c r="G72" s="6"/>
@@ -3703,21 +3712,21 @@
       <c r="J72" s="6"/>
       <c r="K72" s="6"/>
     </row>
-    <row r="73" spans="1:11" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:11" ht="14.55" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A73" s="14">
         <v>72</v>
       </c>
       <c r="B73" s="15" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C73" s="18" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D73" s="19" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E73" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F73" s="7"/>
       <c r="G73" s="8"/>
@@ -3726,21 +3735,21 @@
       <c r="J73" s="8"/>
       <c r="K73" s="8"/>
     </row>
-    <row r="74" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A74" s="9">
         <v>73</v>
       </c>
       <c r="B74" s="12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C74" s="16" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D74" s="17" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E74" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F74" s="3"/>
       <c r="G74" s="6"/>
@@ -3749,21 +3758,21 @@
       <c r="J74" s="6"/>
       <c r="K74" s="6"/>
     </row>
-    <row r="75" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A75" s="9">
         <v>74</v>
       </c>
       <c r="B75" s="13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C75" s="16" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D75" s="17" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E75" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F75" s="3"/>
       <c r="G75" s="6"/>
@@ -3772,21 +3781,21 @@
       <c r="J75" s="6"/>
       <c r="K75" s="6"/>
     </row>
-    <row r="76" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A76" s="9">
         <v>75</v>
       </c>
       <c r="B76" s="13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C76" s="16" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D76" s="17" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E76" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F76" s="3"/>
       <c r="G76" s="6"/>
@@ -3795,21 +3804,21 @@
       <c r="J76" s="6"/>
       <c r="K76" s="6"/>
     </row>
-    <row r="77" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A77" s="9">
         <v>76</v>
       </c>
       <c r="B77" s="13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C77" s="16" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D77" s="17" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E77" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F77" s="2"/>
       <c r="G77" s="6"/>
@@ -3818,21 +3827,21 @@
       <c r="J77" s="6"/>
       <c r="K77" s="6"/>
     </row>
-    <row r="78" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A78" s="9">
         <v>77</v>
       </c>
       <c r="B78" s="13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C78" s="16" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D78" s="17" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E78" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F78" s="3"/>
       <c r="G78" s="6"/>
@@ -3841,21 +3850,21 @@
       <c r="J78" s="6"/>
       <c r="K78" s="6"/>
     </row>
-    <row r="79" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A79" s="9">
         <v>78</v>
       </c>
       <c r="B79" s="13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C79" s="16" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D79" s="17" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E79" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F79" s="3"/>
       <c r="G79" s="6"/>
@@ -3864,21 +3873,21 @@
       <c r="J79" s="6"/>
       <c r="K79" s="6"/>
     </row>
-    <row r="80" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A80" s="9">
         <v>79</v>
       </c>
       <c r="B80" s="13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C80" s="16" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D80" s="17" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E80" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F80" s="3"/>
       <c r="G80" s="6"/>
@@ -3887,21 +3896,21 @@
       <c r="J80" s="6"/>
       <c r="K80" s="6"/>
     </row>
-    <row r="81" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A81" s="9">
         <v>80</v>
       </c>
       <c r="B81" s="13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C81" s="16" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D81" s="17" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E81" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F81" s="3"/>
       <c r="G81" s="6"/>
@@ -3910,21 +3919,21 @@
       <c r="J81" s="6"/>
       <c r="K81" s="6"/>
     </row>
-    <row r="82" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A82" s="9">
         <v>81</v>
       </c>
       <c r="B82" s="13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C82" s="16" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D82" s="17" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E82" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F82" s="3"/>
       <c r="G82" s="6"/>
@@ -3933,21 +3942,21 @@
       <c r="J82" s="6"/>
       <c r="K82" s="6"/>
     </row>
-    <row r="83" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A83" s="9">
         <v>82</v>
       </c>
       <c r="B83" s="13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C83" s="16" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D83" s="17" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E83" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F83" s="3"/>
       <c r="G83" s="6"/>
@@ -3956,21 +3965,21 @@
       <c r="J83" s="6"/>
       <c r="K83" s="6"/>
     </row>
-    <row r="84" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A84" s="9">
         <v>83</v>
       </c>
       <c r="B84" s="13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C84" s="16" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D84" s="17" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E84" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F84" s="3"/>
       <c r="G84" s="6"/>
@@ -3979,21 +3988,21 @@
       <c r="J84" s="6"/>
       <c r="K84" s="6"/>
     </row>
-    <row r="85" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A85" s="9">
         <v>84</v>
       </c>
       <c r="B85" s="13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C85" s="16" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D85" s="17" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E85" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F85" s="3"/>
       <c r="G85" s="6"/>
@@ -4002,21 +4011,21 @@
       <c r="J85" s="6"/>
       <c r="K85" s="6"/>
     </row>
-    <row r="86" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A86" s="9">
         <v>85</v>
       </c>
       <c r="B86" s="13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C86" s="16" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D86" s="17" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E86" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F86" s="3"/>
       <c r="G86" s="6"/>
@@ -4025,21 +4034,21 @@
       <c r="J86" s="6"/>
       <c r="K86" s="6"/>
     </row>
-    <row r="87" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A87" s="9">
         <v>86</v>
       </c>
       <c r="B87" s="13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C87" s="16" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D87" s="17" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E87" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F87" s="3"/>
       <c r="G87" s="6"/>
@@ -4048,21 +4057,21 @@
       <c r="J87" s="6"/>
       <c r="K87" s="6"/>
     </row>
-    <row r="88" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A88" s="9">
         <v>87</v>
       </c>
       <c r="B88" s="13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C88" s="16" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D88" s="17" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E88" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F88" s="3"/>
       <c r="G88" s="6"/>
@@ -4071,21 +4080,21 @@
       <c r="J88" s="6"/>
       <c r="K88" s="6"/>
     </row>
-    <row r="89" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A89" s="9">
         <v>88</v>
       </c>
       <c r="B89" s="13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C89" s="16" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D89" s="17" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="E89" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F89" s="3"/>
       <c r="G89" s="6"/>
@@ -4094,21 +4103,21 @@
       <c r="J89" s="6"/>
       <c r="K89" s="6"/>
     </row>
-    <row r="90" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A90" s="9">
         <v>89</v>
       </c>
       <c r="B90" s="13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C90" s="16" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D90" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E90" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F90" s="3"/>
       <c r="G90" s="6"/>
@@ -4117,21 +4126,21 @@
       <c r="J90" s="6"/>
       <c r="K90" s="6"/>
     </row>
-    <row r="91" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A91" s="9">
         <v>90</v>
       </c>
       <c r="B91" s="13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C91" s="16" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D91" s="17" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E91" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F91" s="3"/>
       <c r="G91" s="6"/>
@@ -4140,21 +4149,21 @@
       <c r="J91" s="6"/>
       <c r="K91" s="6"/>
     </row>
-    <row r="92" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A92" s="9">
         <v>91</v>
       </c>
       <c r="B92" s="13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C92" s="16" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D92" s="17" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="E92" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F92" s="3"/>
       <c r="G92" s="6"/>
@@ -4163,21 +4172,21 @@
       <c r="J92" s="6"/>
       <c r="K92" s="6"/>
     </row>
-    <row r="93" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A93" s="9">
         <v>92</v>
       </c>
       <c r="B93" s="13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C93" s="16" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D93" s="17" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E93" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F93" s="3"/>
       <c r="G93" s="6"/>
@@ -4186,21 +4195,21 @@
       <c r="J93" s="6"/>
       <c r="K93" s="6"/>
     </row>
-    <row r="94" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A94" s="9">
         <v>93</v>
       </c>
       <c r="B94" s="13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C94" s="16" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D94" s="17" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E94" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F94" s="3"/>
       <c r="G94" s="6"/>
@@ -4209,21 +4218,21 @@
       <c r="J94" s="6"/>
       <c r="K94" s="6"/>
     </row>
-    <row r="95" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A95" s="9">
         <v>94</v>
       </c>
       <c r="B95" s="13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C95" s="16" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D95" s="16" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="E95" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F95" s="3"/>
       <c r="G95" s="6"/>
@@ -4232,21 +4241,21 @@
       <c r="J95" s="6"/>
       <c r="K95" s="6"/>
     </row>
-    <row r="96" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A96" s="9">
         <v>95</v>
       </c>
       <c r="B96" s="13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C96" s="16" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D96" s="16" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="E96" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F96" s="3"/>
       <c r="G96" s="6"/>
@@ -4255,21 +4264,21 @@
       <c r="J96" s="6"/>
       <c r="K96" s="6"/>
     </row>
-    <row r="97" spans="1:11" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:11" ht="14.55" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A97" s="14">
         <v>96</v>
       </c>
       <c r="B97" s="15" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C97" s="18" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D97" s="19" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E97" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F97" s="7"/>
       <c r="G97" s="8"/>
@@ -4278,28 +4287,28 @@
       <c r="J97" s="8"/>
       <c r="K97" s="8"/>
     </row>
-    <row r="145" spans="4:4" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="4:4" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="D145" s="5"/>
     </row>
-    <row r="146" spans="4:4" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="4:4" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="D146" s="5"/>
     </row>
-    <row r="147" spans="4:4" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="4:4" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="D147" s="5"/>
     </row>
-    <row r="148" spans="4:4" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="4:4" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="D148" s="5"/>
     </row>
-    <row r="170" spans="4:4" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="4:4" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="D170" s="5"/>
     </row>
-    <row r="171" spans="4:4" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="4:4" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="D171" s="5"/>
     </row>
-    <row r="172" spans="4:4" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="4:4" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="D172" s="5"/>
     </row>
-    <row r="173" spans="4:4" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="4:4" ht="14.55" customHeight="1" x14ac:dyDescent="0.4">
       <c r="D173" s="5"/>
     </row>
   </sheetData>
@@ -4309,65 +4318,22 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_dlc_DocId xmlns="fa7e5010-1311-4096-a344-326d1919664c">JFHTZT72FDVU-254938863-279</_dlc_DocId>
+    <_dlc_DocIdUrl xmlns="fa7e5010-1311-4096-a344-326d1919664c">
+      <Url>https://intranet.d-fine.de/intern/miscellaneous/TemplateFramework/_layouts/15/DocIdRedir.aspx?ID=JFHTZT72FDVU-254938863-279</Url>
+      <Description>JFHTZT72FDVU-254938863-279</Description>
+    </_dlc_DocIdUrl>
+    <_Version xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <Tools xmlns="255ceb00-0504-4451-971c-89cf8ee3ad27"/>
+    <Comments xmlns="255ceb00-0504-4451-971c-89cf8ee3ad27" xsi:nil="true"/>
+    <Document_x0020_Category xmlns="255ceb00-0504-4451-971c-89cf8ee3ad27"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=15.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=15.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=15.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=15.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100135AEE51B13C7A4784C7A6FB658DD0E0" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c2ccf66da846160ccad12796df698db1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="fa7e5010-1311-4096-a344-326d1919664c" xmlns:ns3="http://schemas.microsoft.com/sharepoint/v3/fields" xmlns:ns4="255ceb00-0504-4451-971c-89cf8ee3ad27" xmlns:ns5="953edb04-63dd-49ba-ad7b-e9d17e0e7f06" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="cd9e9067e801230649229059a2f6238c" ns2:_="" ns3:_="" ns4:_="" ns5:_="">
     <xsd:import namespace="fa7e5010-1311-4096-a344-326d1919664c"/>
@@ -4613,39 +4579,85 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=15.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=15.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=15.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=15.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
+</file>
+
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_dlc_DocId xmlns="fa7e5010-1311-4096-a344-326d1919664c">JFHTZT72FDVU-254938863-279</_dlc_DocId>
-    <_dlc_DocIdUrl xmlns="fa7e5010-1311-4096-a344-326d1919664c">
-      <Url>https://intranet.d-fine.de/intern/miscellaneous/TemplateFramework/_layouts/15/DocIdRedir.aspx?ID=JFHTZT72FDVU-254938863-279</Url>
-      <Description>JFHTZT72FDVU-254938863-279</Description>
-    </_dlc_DocIdUrl>
-    <_Version xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <Tools xmlns="255ceb00-0504-4451-971c-89cf8ee3ad27"/>
-    <Comments xmlns="255ceb00-0504-4451-971c-89cf8ee3ad27" xsi:nil="true"/>
-    <Document_x0020_Category xmlns="255ceb00-0504-4451-971c-89cf8ee3ad27"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB0B7321-043A-43C5-BAA4-E29877D5579D}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7017BB2C-A3F1-4167-848C-B358A8DC1CB9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="fa7e5010-1311-4096-a344-326d1919664c"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="255ceb00-0504-4451-971c-89cf8ee3ad27"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="953edb04-63dd-49ba-ad7b-e9d17e0e7f06"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{27E0ED53-E837-41F7-A9C9-5E67E49390EA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FF6E80A2-72F6-4920-8A44-B99818E21D00}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4666,21 +4678,18 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{27E0ED53-E837-41F7-A9C9-5E67E49390EA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7017BB2C-A3F1-4167-848C-B358A8DC1CB9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB0B7321-043A-43C5-BAA4-E29877D5579D}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="fa7e5010-1311-4096-a344-326d1919664c"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="255ceb00-0504-4451-971c-89cf8ee3ad27"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="953edb04-63dd-49ba-ad7b-e9d17e0e7f06"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>